<commit_message>
Did pp data collection
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60799752-090D-4C1D-A7E9-24751C8ED924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0352308F-A230-49B5-B522-09B8FC0947B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6540" yWindow="1905" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1560" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -63,13 +63,13 @@
     <t>cs</t>
   </si>
   <si>
-    <t>GPU</t>
-  </si>
-  <si>
     <t>multi</t>
   </si>
   <si>
     <t>PC 1</t>
+  </si>
+  <si>
+    <t>shaders</t>
   </si>
 </sst>
 </file>
@@ -192,10 +192,10 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
@@ -494,7 +494,7 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
@@ -547,6 +547,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="5"/>
+      <c r="H7" s="9"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
@@ -558,6 +559,7 @@
       <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="H8" s="9"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
@@ -636,7 +638,7 @@
         <v>4</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
@@ -676,7 +678,7 @@
         <v>4</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
More pp data collection ... i think theres only quick data collections left
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0352308F-A230-49B5-B522-09B8FC0947B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C8982F-8FAB-494B-A2F9-69E7306069D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1950" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="2910" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -527,6 +527,7 @@
       </c>
       <c r="D5" s="5"/>
       <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
       <c r="H5" s="9"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
@@ -537,6 +538,8 @@
         <v>5</v>
       </c>
       <c r="D6" s="5"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
       <c r="H6" s="9"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Did cs data collection for 800 and 1600
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3C8982F-8FAB-494B-A2F9-69E7306069D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A476BCC7-A491-48F4-B26F-BA19C9AE1BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2910" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4425" yWindow="2565" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -644,7 +644,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>11</v>
       </c>
@@ -652,8 +652,10 @@
         <v>4</v>
       </c>
       <c r="D17" s="8"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>11</v>
       </c>
@@ -661,8 +663,10 @@
         <v>6</v>
       </c>
       <c r="D18" s="8"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>11</v>
       </c>
@@ -672,8 +676,10 @@
       <c r="D19" s="8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>11</v>
       </c>
@@ -683,6 +689,8 @@
       <c r="D20" s="8" t="s">
         <v>14</v>
       </c>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Did final cs and most of cr data collection
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A476BCC7-A491-48F4-B26F-BA19C9AE1BE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ABBFB47-EE7B-4D8E-AA11-E7AC39654672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4425" yWindow="2565" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6870" yWindow="2535" windowWidth="17565" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -491,6 +491,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:H20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="8" customWidth="1"/>
+    <col min="7" max="8" width="9.140625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="11" t="s">
@@ -601,6 +605,8 @@
         <v>4</v>
       </c>
       <c r="D12" s="7"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
@@ -610,6 +616,8 @@
         <v>6</v>
       </c>
       <c r="D13" s="7"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
@@ -621,6 +629,8 @@
       <c r="D14" s="7" t="s">
         <v>7</v>
       </c>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
@@ -632,6 +642,8 @@
       <c r="D15" s="7" t="s">
         <v>10</v>
       </c>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
@@ -643,6 +655,8 @@
       <c r="D16" s="7" t="s">
         <v>12</v>
       </c>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
@@ -652,6 +666,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="8"/>
+      <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
     </row>
@@ -663,6 +678,7 @@
         <v>6</v>
       </c>
       <c r="D18" s="8"/>
+      <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
     </row>
@@ -676,6 +692,7 @@
       <c r="D19" s="8" t="s">
         <v>7</v>
       </c>
+      <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="9"/>
     </row>
@@ -689,6 +706,7 @@
       <c r="D20" s="8" t="s">
         <v>14</v>
       </c>
+      <c r="F20" s="9"/>
       <c r="G20" s="9"/>
       <c r="H20" s="9"/>
     </row>

</xml_diff>

<commit_message>
Did more cr and pp data collection
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ABBFB47-EE7B-4D8E-AA11-E7AC39654672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF48409C-1560-402C-ADAF-B3675DB37934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6870" yWindow="2535" windowWidth="17565" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8880" yWindow="2925" windowWidth="17565" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -554,6 +554,8 @@
         <v>6</v>
       </c>
       <c r="D7" s="5"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
       <c r="H7" s="9"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
@@ -566,6 +568,8 @@
       <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
       <c r="H8" s="9"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
@@ -607,6 +611,7 @@
       <c r="D12" s="7"/>
       <c r="F12" s="9"/>
       <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
@@ -618,6 +623,7 @@
       <c r="D13" s="7"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
@@ -631,6 +637,7 @@
       </c>
       <c r="F14" s="9"/>
       <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
@@ -644,6 +651,7 @@
       </c>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
@@ -657,6 +665,7 @@
       </c>
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">

</xml_diff>

<commit_message>
Started js data collection
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF48409C-1560-402C-ADAF-B3675DB37934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A00D5B-4012-454B-A17F-14450B8F6CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8880" yWindow="2925" windowWidth="17565" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -200,9 +200,12 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,28 +500,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10">
+      <c r="E3" s="9"/>
+      <c r="F3" s="9">
         <v>400</v>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="9">
         <v>800</v>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="9">
         <v>1600</v>
       </c>
     </row>
@@ -530,9 +533,9 @@
         <v>4</v>
       </c>
       <c r="D5" s="5"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
@@ -542,9 +545,9 @@
         <v>5</v>
       </c>
       <c r="D6" s="5"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
@@ -554,9 +557,9 @@
         <v>6</v>
       </c>
       <c r="D7" s="5"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
@@ -568,9 +571,9 @@
       <c r="D8" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
@@ -580,6 +583,9 @@
         <v>4</v>
       </c>
       <c r="D9" s="6"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
@@ -589,6 +595,9 @@
         <v>6</v>
       </c>
       <c r="D10" s="6"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
@@ -600,6 +609,9 @@
       <c r="D11" s="6" t="s">
         <v>7</v>
       </c>
+      <c r="F11" s="13"/>
+      <c r="G11" s="14"/>
+      <c r="H11" s="14"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
@@ -609,9 +621,9 @@
         <v>4</v>
       </c>
       <c r="D12" s="7"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
     </row>
     <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
@@ -621,9 +633,9 @@
         <v>6</v>
       </c>
       <c r="D13" s="7"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
@@ -635,9 +647,9 @@
       <c r="D14" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
     </row>
     <row r="15" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
@@ -649,9 +661,9 @@
       <c r="D15" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B16" s="3" t="s">
@@ -663,9 +675,9 @@
       <c r="D16" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
@@ -675,9 +687,9 @@
         <v>4</v>
       </c>
       <c r="D17" s="8"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
@@ -687,9 +699,9 @@
         <v>6</v>
       </c>
       <c r="D18" s="8"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
@@ -701,9 +713,9 @@
       <c r="D19" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
@@ -715,9 +727,9 @@
       <c r="D20" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finished main data collection
</commit_message>
<xml_diff>
--- a/Source/DataProccessing/Data_V1.2/collected.xlsx
+++ b/Source/DataProccessing/Data_V1.2/collected.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Projects\FastCGOL_prjct\FastCGOL\Source\DataProccessing\Data_V1.2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63A00D5B-4012-454B-A17F-14450B8F6CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E78E94-2DEB-45B4-A355-48EAD065E5D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8880" yWindow="2925" windowWidth="17565" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6840" yWindow="1485" windowWidth="15270" windowHeight="11865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -202,10 +202,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,9 +580,9 @@
         <v>4</v>
       </c>
       <c r="D9" s="6"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
@@ -595,9 +592,9 @@
         <v>6</v>
       </c>
       <c r="D10" s="6"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
@@ -609,9 +606,9 @@
       <c r="D11" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="14"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">

</xml_diff>